<commit_message>
Correct basketball TOV% definition and add raw box-score data
Recompute TOV% as TOV/possessions (matching the study's stated definition)
rather than the Kubatko TOV/(FGA+0.44*FTA+TOV) form the tidy file previously
carried. Adds fiba_wc_2023_boxscores.xlsx with the underlying raw totals and
documents every indicator formula in the README so the four medal-round teams'
Four Factors are fully reproducible.
</commit_message>
<xml_diff>
--- a/FIBA_WC_2023.xlsx
+++ b/FIBA_WC_2023.xlsx
@@ -504,7 +504,7 @@
         <v>0.3488</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1054</v>
+        <v>0.1252</v>
       </c>
       <c r="I2" t="n">
         <v>0.274</v>
@@ -539,7 +539,7 @@
         <v>0.5238</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1645</v>
+        <v>0.187</v>
       </c>
       <c r="I3" t="n">
         <v>0.1429</v>
@@ -574,7 +574,7 @@
         <v>0.3824</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0873</v>
+        <v>0.1017</v>
       </c>
       <c r="I4" t="n">
         <v>0.1486</v>
@@ -609,7 +609,7 @@
         <v>0.3</v>
       </c>
       <c r="H5" t="n">
-        <v>0.09030000000000001</v>
+        <v>0.1069</v>
       </c>
       <c r="I5" t="n">
         <v>0.2381</v>
@@ -644,7 +644,7 @@
         <v>0.2609</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1707</v>
+        <v>0.1842</v>
       </c>
       <c r="I6" t="n">
         <v>0.3684</v>
@@ -679,7 +679,7 @@
         <v>0.3667</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1169</v>
+        <v>0.1342</v>
       </c>
       <c r="I7" t="n">
         <v>0.4426</v>
@@ -714,7 +714,7 @@
         <v>0.2308</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1607</v>
+        <v>0.1736</v>
       </c>
       <c r="I8" t="n">
         <v>0.3929</v>
@@ -749,7 +749,7 @@
         <v>0.2821</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1025</v>
+        <v>0.1142</v>
       </c>
       <c r="I9" t="n">
         <v>0.2857</v>
@@ -784,7 +784,7 @@
         <v>0.2727</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1163</v>
+        <v>0.1299</v>
       </c>
       <c r="I10" t="n">
         <v>0.09719999999999999</v>
@@ -819,7 +819,7 @@
         <v>0.1852</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1508</v>
+        <v>0.1609</v>
       </c>
       <c r="I11" t="n">
         <v>0.1967</v>
@@ -854,7 +854,7 @@
         <v>0.3913</v>
       </c>
       <c r="H12" t="n">
-        <v>0.0853</v>
+        <v>0.0959</v>
       </c>
       <c r="I12" t="n">
         <v>0.1765</v>
@@ -889,7 +889,7 @@
         <v>0.2414</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1294</v>
+        <v>0.141</v>
       </c>
       <c r="I13" t="n">
         <v>0.2222</v>
@@ -924,7 +924,7 @@
         <v>0.3333</v>
       </c>
       <c r="H14" t="n">
-        <v>0.1539</v>
+        <v>0.1722</v>
       </c>
       <c r="I14" t="n">
         <v>0.2344</v>
@@ -959,7 +959,7 @@
         <v>0.3333</v>
       </c>
       <c r="H15" t="n">
-        <v>0.0926</v>
+        <v>0.109</v>
       </c>
       <c r="I15" t="n">
         <v>0.2429</v>
@@ -994,7 +994,7 @@
         <v>0.2857</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1103</v>
+        <v>0.1209</v>
       </c>
       <c r="I16" t="n">
         <v>0.2535</v>
@@ -1029,7 +1029,7 @@
         <v>0.36</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1646</v>
+        <v>0.1857</v>
       </c>
       <c r="I17" t="n">
         <v>0.4</v>
@@ -1064,7 +1064,7 @@
         <v>0.2222</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1336</v>
+        <v>0.1442</v>
       </c>
       <c r="I18" t="n">
         <v>0.4068</v>
@@ -1099,7 +1099,7 @@
         <v>0.2667</v>
       </c>
       <c r="H19" t="n">
-        <v>0.1261</v>
+        <v>0.1389</v>
       </c>
       <c r="I19" t="n">
         <v>0.2388</v>
@@ -1134,7 +1134,7 @@
         <v>0.3636</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0958</v>
+        <v>0.106</v>
       </c>
       <c r="I20" t="n">
         <v>0.2059</v>
@@ -1169,7 +1169,7 @@
         <v>0.2286</v>
       </c>
       <c r="H21" t="n">
-        <v>0.1218</v>
+        <v>0.135</v>
       </c>
       <c r="I21" t="n">
         <v>0.4655</v>
@@ -1204,7 +1204,7 @@
         <v>0.2105</v>
       </c>
       <c r="H22" t="n">
-        <v>0.1149</v>
+        <v>0.1205</v>
       </c>
       <c r="I22" t="n">
         <v>0.2727</v>
@@ -1239,7 +1239,7 @@
         <v>0.3077</v>
       </c>
       <c r="H23" t="n">
-        <v>0.0934</v>
+        <v>0.1046</v>
       </c>
       <c r="I23" t="n">
         <v>0.2</v>
@@ -1274,7 +1274,7 @@
         <v>0.3</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1834</v>
+        <v>0.1979</v>
       </c>
       <c r="I24" t="n">
         <v>0.2414</v>
@@ -1309,7 +1309,7 @@
         <v>0.3226</v>
       </c>
       <c r="H25" t="n">
-        <v>0.1244</v>
+        <v>0.142</v>
       </c>
       <c r="I25" t="n">
         <v>0.2581</v>
@@ -1344,7 +1344,7 @@
         <v>0.2174</v>
       </c>
       <c r="H26" t="n">
-        <v>0.2114</v>
+        <v>0.2238</v>
       </c>
       <c r="I26" t="n">
         <v>0.3559</v>
@@ -1414,7 +1414,7 @@
         <v>0.3415</v>
       </c>
       <c r="H28" t="n">
-        <v>0.1317</v>
+        <v>0.1517</v>
       </c>
       <c r="I28" t="n">
         <v>0.275</v>
@@ -1449,7 +1449,7 @@
         <v>0.2353</v>
       </c>
       <c r="H29" t="n">
-        <v>0.1361</v>
+        <v>0.1496</v>
       </c>
       <c r="I29" t="n">
         <v>0.3175</v>
@@ -1484,7 +1484,7 @@
         <v>0.2333</v>
       </c>
       <c r="H30" t="n">
-        <v>0.1191</v>
+        <v>0.1288</v>
       </c>
       <c r="I30" t="n">
         <v>0.2055</v>
@@ -1554,7 +1554,7 @@
         <v>0.25</v>
       </c>
       <c r="H32" t="n">
-        <v>0.1064</v>
+        <v>0.1145</v>
       </c>
       <c r="I32" t="n">
         <v>0.3538</v>
@@ -1589,7 +1589,7 @@
         <v>0.3158</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1283</v>
+        <v>0.1442</v>
       </c>
       <c r="I33" t="n">
         <v>0.2963</v>

</xml_diff>

<commit_message>
Correct basketball DEFRTG definition (opponent points per opponent possession)
DEFRTG is a team's points allowed divided by the opponent's possessions
(i.e. the opponent's offensive rating), not points allowed over the team's own
possessions. Recomputing this reproduces the published Table 3 DEFRTG values
and Table 4 slopes exactly (e.g. Canada DEFRTG beta=1.06, R2=0.85).
</commit_message>
<xml_diff>
--- a/FIBA_WC_2023.xlsx
+++ b/FIBA_WC_2023.xlsx
@@ -495,7 +495,7 @@
         <v>118.9</v>
       </c>
       <c r="E2" t="n">
-        <v>81.40000000000001</v>
+        <v>84.7</v>
       </c>
       <c r="F2" t="n">
         <v>0.5137</v>
@@ -530,7 +530,7 @@
         <v>159.7</v>
       </c>
       <c r="E3" t="n">
-        <v>91.09999999999999</v>
+        <v>91</v>
       </c>
       <c r="F3" t="n">
         <v>0.8429</v>
@@ -565,7 +565,7 @@
         <v>128.4</v>
       </c>
       <c r="E4" t="n">
-        <v>95.3</v>
+        <v>98.3</v>
       </c>
       <c r="F4" t="n">
         <v>0.6081</v>
@@ -600,7 +600,7 @@
         <v>99.3</v>
       </c>
       <c r="E5" t="n">
-        <v>105.4</v>
+        <v>106.2</v>
       </c>
       <c r="F5" t="n">
         <v>0.3968</v>
@@ -635,7 +635,7 @@
         <v>115.8</v>
       </c>
       <c r="E6" t="n">
-        <v>111.8</v>
+        <v>112.1</v>
       </c>
       <c r="F6" t="n">
         <v>0.5877</v>
@@ -670,7 +670,7 @@
         <v>134.2</v>
       </c>
       <c r="E7" t="n">
-        <v>119.4</v>
+        <v>118</v>
       </c>
       <c r="F7" t="n">
         <v>0.5984</v>
@@ -705,7 +705,7 @@
         <v>114.9</v>
       </c>
       <c r="E8" t="n">
-        <v>126.9</v>
+        <v>125.3</v>
       </c>
       <c r="F8" t="n">
         <v>0.5714</v>
@@ -740,7 +740,7 @@
         <v>131.9</v>
       </c>
       <c r="E9" t="n">
-        <v>122.5</v>
+        <v>121.5</v>
       </c>
       <c r="F9" t="n">
         <v>0.6131</v>
@@ -775,7 +775,7 @@
         <v>105.2</v>
       </c>
       <c r="E10" t="n">
-        <v>81.90000000000001</v>
+        <v>80.3</v>
       </c>
       <c r="F10" t="n">
         <v>0.5139</v>
@@ -810,7 +810,7 @@
         <v>113.9</v>
       </c>
       <c r="E11" t="n">
-        <v>109.9</v>
+        <v>113.9</v>
       </c>
       <c r="F11" t="n">
         <v>0.5984</v>
@@ -845,7 +845,7 @@
         <v>138.3</v>
       </c>
       <c r="E12" t="n">
-        <v>102.7</v>
+        <v>107.9</v>
       </c>
       <c r="F12" t="n">
         <v>0.6544</v>
@@ -880,7 +880,7 @@
         <v>128.2</v>
       </c>
       <c r="E13" t="n">
-        <v>93.59999999999999</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="F13" t="n">
         <v>0.6825</v>
@@ -915,7 +915,7 @@
         <v>132.5</v>
       </c>
       <c r="E14" t="n">
-        <v>94.09999999999999</v>
+        <v>92</v>
       </c>
       <c r="F14" t="n">
         <v>0.6641</v>
@@ -950,7 +950,7 @@
         <v>110.4</v>
       </c>
       <c r="E15" t="n">
-        <v>107.7</v>
+        <v>107.6</v>
       </c>
       <c r="F15" t="n">
         <v>0.4571</v>
@@ -985,7 +985,7 @@
         <v>136.7</v>
       </c>
       <c r="E16" t="n">
-        <v>134.3</v>
+        <v>141.2</v>
       </c>
       <c r="F16" t="n">
         <v>0.669</v>
@@ -1020,7 +1020,7 @@
         <v>118.6</v>
       </c>
       <c r="E17" t="n">
-        <v>110</v>
+        <v>109.4</v>
       </c>
       <c r="F17" t="n">
         <v>0.5545</v>
@@ -1055,7 +1055,7 @@
         <v>137.6</v>
       </c>
       <c r="E18" t="n">
-        <v>82.5</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="F18" t="n">
         <v>0.6864</v>
@@ -1090,7 +1090,7 @@
         <v>118.6</v>
       </c>
       <c r="E19" t="n">
-        <v>97.2</v>
+        <v>96.2</v>
       </c>
       <c r="F19" t="n">
         <v>0.5821</v>
@@ -1125,7 +1125,7 @@
         <v>152.4</v>
       </c>
       <c r="E20" t="n">
-        <v>110</v>
+        <v>107.8</v>
       </c>
       <c r="F20" t="n">
         <v>0.7426</v>
@@ -1160,7 +1160,7 @@
         <v>102.6</v>
       </c>
       <c r="E21" t="n">
-        <v>105.3</v>
+        <v>106</v>
       </c>
       <c r="F21" t="n">
         <v>0.4224</v>
@@ -1195,7 +1195,7 @@
         <v>134.9</v>
       </c>
       <c r="E22" t="n">
-        <v>95.2</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="F22" t="n">
         <v>0.7121</v>
@@ -1230,7 +1230,7 @@
         <v>130</v>
       </c>
       <c r="E23" t="n">
-        <v>101.6</v>
+        <v>100.6</v>
       </c>
       <c r="F23" t="n">
         <v>0.625</v>
@@ -1265,7 +1265,7 @@
         <v>125.3</v>
       </c>
       <c r="E24" t="n">
-        <v>113.5</v>
+        <v>114.8</v>
       </c>
       <c r="F24" t="n">
         <v>0.6983</v>
@@ -1300,7 +1300,7 @@
         <v>109.4</v>
       </c>
       <c r="E25" t="n">
-        <v>118</v>
+        <v>118.6</v>
       </c>
       <c r="F25" t="n">
         <v>0.4919</v>
@@ -1335,7 +1335,7 @@
         <v>116.6</v>
       </c>
       <c r="E26" t="n">
-        <v>84.8</v>
+        <v>79.7</v>
       </c>
       <c r="F26" t="n">
         <v>0.661</v>
@@ -1370,7 +1370,7 @@
         <v>141.6</v>
       </c>
       <c r="E27" t="n">
-        <v>105.2</v>
+        <v>98.8</v>
       </c>
       <c r="F27" t="n">
         <v>0.6475</v>
@@ -1405,7 +1405,7 @@
         <v>119.2</v>
       </c>
       <c r="E28" t="n">
-        <v>67.2</v>
+        <v>69.3</v>
       </c>
       <c r="F28" t="n">
         <v>0.55</v>
@@ -1440,7 +1440,7 @@
         <v>106</v>
       </c>
       <c r="E29" t="n">
-        <v>91</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="F29" t="n">
         <v>0.5159</v>
@@ -1475,7 +1475,7 @@
         <v>121.8</v>
       </c>
       <c r="E30" t="n">
-        <v>128.9</v>
+        <v>129.4</v>
       </c>
       <c r="F30" t="n">
         <v>0.6096</v>
@@ -1510,7 +1510,7 @@
         <v>118.2</v>
       </c>
       <c r="E31" t="n">
-        <v>74.5</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="F31" t="n">
         <v>0.6642</v>
@@ -1545,7 +1545,7 @@
         <v>141.3</v>
       </c>
       <c r="E32" t="n">
-        <v>143.8</v>
+        <v>136.6</v>
       </c>
       <c r="F32" t="n">
         <v>0.6768999999999999</v>
@@ -1580,7 +1580,7 @@
         <v>121.5</v>
       </c>
       <c r="E33" t="n">
-        <v>130.8</v>
+        <v>131.9</v>
       </c>
       <c r="F33" t="n">
         <v>0.5802</v>

</xml_diff>